<commit_message>
Fix generator selection for misindexed permits
</commit_message>
<xml_diff>
--- a/processed-data/illinois-data-center-regulatory-inventory.xlsx
+++ b/processed-data/illinois-data-center-regulatory-inventory.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facilities" sheetId="1" r:id="R7271e09cbc9e4535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="R049b86d75e0440cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generators" sheetId="3" r:id="Ra3cdc6b52de54528"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Permits and Limits" sheetId="4" r:id="R9898e51155204f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="5" r:id="R41826b906f1c43ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facilities" sheetId="1" r:id="R1c8235f58f584ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="R6fff2d6aa6784e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generators" sheetId="3" r:id="Rc91474a83fee4588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Permits and Limits" sheetId="4" r:id="R91783f08704245b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="5" r:id="Rff76827897304fe6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -263,8 +263,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GeneratorsTable" displayName="GeneratorsTable" ref="A1:U39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:U39"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GeneratorsTable" displayName="GeneratorsTable" ref="A1:U42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:U42"/>
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="Generator Record ID"/>
     <x:tableColumn id="2" name="Facility IDs"/>
@@ -671,13 +671,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="P2" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Q2" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="R2" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>19500</x:v>
       </x:c>
       <x:c r="S2" s="14" t="str">
         <x:v>Equinix LLC</x:v>
@@ -1966,7 +1966,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8350ede8fba24380"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf1f489dad014668"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7919,7 +7919,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8efbc1fa744c74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R649757341be14cac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8018,19 +8018,19 @@
     </x:row>
     <x:row r="2" ht="31.5" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>GEN-DOC-170000341994-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170000063561-AIR-003-01</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
-        <x:v>IL_N_2</x:v>
+        <x:v>IL_N_1</x:v>
       </x:c>
       <x:c r="C2" s="15" t="str">
-        <x:v>170000341994</x:v>
+        <x:v>170000063561</x:v>
       </x:c>
       <x:c r="D2" s="13" t="str">
-        <x:v>DOC-170000341994-AIR-001</x:v>
+        <x:v>DOC-170000063561-AIR-003</x:v>
       </x:c>
       <x:c r="E2" s="18" t="n">
-        <x:v>44348</x:v>
+        <x:v>45357</x:v>
       </x:c>
       <x:c r="F2" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8039,20 +8039,20 @@
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H2" s="14" t="str">
-        <x:v>Generator #7</x:v>
+        <x:v>G-1 thru G-6</x:v>
       </x:c>
       <x:c r="I2" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J2" s="17" t="n">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="K2" s="17" t="n">
         <x:f>IF(OR(I2="",J2=""),"",I2*J2)</x:f>
-        <x:v>1500</x:v>
+        <x:v>9000</x:v>
       </x:c>
       <x:c r="L2" s="17" t="n">
-        <x:v>2139</x:v>
+        <x:v>2153</x:v>
       </x:c>
       <x:c r="M2" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8063,7 +8063,7 @@
         <x:v>Permitted / described</x:v>
       </x:c>
       <x:c r="Q2" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="R2" s="14" t="str">
         <x:v>OCR pattern extraction</x:v>
@@ -8072,27 +8072,27 @@
         <x:v>OCR extracted - review recommended</x:v>
       </x:c>
       <x:c r="T2" s="13" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="U2" s="14" t="str">
-        <x:v>Description of emission units to be operated: 1,500 KW (2,139 hp) Diesel Fueled Emergency Generator (Generator #7) Mail check and/or form to Illinols EPA, BOA-Permit Section, 1021 North Grand Ave. Ea</x:v>
+        <x:v>ated Permittee to OPERATE emission source (s) and/or air pollution control equipment consisting of: Six (6) 1,500 kw (2,153 HP) diesel-powered emergency engine/generators (G-1 thru G-6) Four (4) 2,000 kW (2,897 HP) diesel-powered emergency engine/generators (...</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="31.5" customHeight="1">
       <x:c r="A3" s="13" t="str">
-        <x:v>GEN-DOC-170001699320-AIR-002-01</x:v>
+        <x:v>GEN-DOC-170000063561-AIR-003-02</x:v>
       </x:c>
       <x:c r="B3" s="13" t="str">
-        <x:v>IL_N_23</x:v>
+        <x:v>IL_N_1</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>170001699320</x:v>
+        <x:v>170000063561</x:v>
       </x:c>
       <x:c r="D3" s="13" t="str">
-        <x:v>DOC-170001699320-AIR-002</x:v>
+        <x:v>DOC-170000063561-AIR-003</x:v>
       </x:c>
       <x:c r="E3" s="18" t="n">
-        <x:v>40420</x:v>
+        <x:v>45357</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8100,18 +8100,22 @@
       <x:c r="G3" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H3" s="14"/>
+      <x:c r="H3" s="14" t="str">
+        <x:v>G-7</x:v>
+      </x:c>
       <x:c r="I3" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J3" s="17" t="n">
         <x:v>2000</x:v>
       </x:c>
       <x:c r="K3" s="17" t="n">
         <x:f>IF(OR(I3="",J3=""),"",I3*J3)</x:f>
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="L3" s="17"/>
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="L3" s="17" t="n">
+        <x:v>2897</x:v>
+      </x:c>
       <x:c r="M3" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -8133,24 +8137,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U3" s="14" t="str">
-        <x:v>ignated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of three 2,000 kW. (two (2) 2,876-HP and one (1) 3,937-HP) #2 fuel oil fired emergency generators</x:v>
+        <x:v>onsisting of: Six (6) 1,500 kw (2,153 HP) diesel-powered emergency engine/generators (G-1 thru G-6) Four (4) 2,000 kW (2,897 HP) diesel-powered emergency engine/generators (G-7 G-10) thru (1) 2,500 kW (3,633 HP) diesel-powered emergency engine/generator (G-11)</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="31.5" customHeight="1">
       <x:c r="A4" s="13" t="str">
-        <x:v>GEN-DOC-170001764240-AIR-005-01</x:v>
+        <x:v>GEN-DOC-170000063561-AIR-003-03</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>IL_N_4</x:v>
+        <x:v>IL_N_1</x:v>
       </x:c>
       <x:c r="C4" s="15" t="str">
-        <x:v>170001764240</x:v>
+        <x:v>170000063561</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
-        <x:v>DOC-170001764240-AIR-005</x:v>
+        <x:v>DOC-170000063561-AIR-003</x:v>
       </x:c>
       <x:c r="E4" s="18" t="n">
-        <x:v>44167</x:v>
+        <x:v>45357</x:v>
       </x:c>
       <x:c r="F4" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8158,19 +8162,21 @@
       <x:c r="G4" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H4" s="14"/>
+      <x:c r="H4" s="14" t="str">
+        <x:v>G-11</x:v>
+      </x:c>
       <x:c r="I4" s="17" t="n">
-        <x:v>11</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="17" t="n">
-        <x:v>2740</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="K4" s="17" t="n">
         <x:f>IF(OR(I4="",J4=""),"",I4*J4)</x:f>
-        <x:v>30140</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="L4" s="17" t="n">
-        <x:v>3673</x:v>
+        <x:v>3633</x:v>
       </x:c>
       <x:c r="M4" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8193,24 +8199,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U4" s="14" t="str">
-        <x:v>ignated Permittee to OPERATE and/or air pollution control equipment consisting of emission unit (s) Eleven (11) 2,740 kw (3,673 engine HP) diesel-powered emergency generator sets; Seventeen (17) 3,490 kW (4,678 engine HP) diesel-powered emergency generator se...</x:v>
+        <x:v>1 thru G-6) Four (4) 2,000 kW (2,897 HP) diesel-powered emergency engine/generators (G-7 G-10) thru (1) 2,500 kW (3,633 HP) diesel-powered emergency engine/generator (G-11)</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="31.5" customHeight="1">
       <x:c r="A5" s="13" t="str">
-        <x:v>GEN-DOC-170001764240-AIR-005-02</x:v>
+        <x:v>GEN-DOC-170000341994-AIR-001-01</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>IL_N_4</x:v>
+        <x:v>IL_N_2</x:v>
       </x:c>
       <x:c r="C5" s="15" t="str">
-        <x:v>170001764240</x:v>
+        <x:v>170000341994</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
-        <x:v>DOC-170001764240-AIR-005</x:v>
+        <x:v>DOC-170000341994-AIR-001</x:v>
       </x:c>
       <x:c r="E5" s="18" t="n">
-        <x:v>44167</x:v>
+        <x:v>44348</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8218,19 +8224,21 @@
       <x:c r="G5" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H5" s="14"/>
+      <x:c r="H5" s="14" t="str">
+        <x:v>Generator #7</x:v>
+      </x:c>
       <x:c r="I5" s="17" t="n">
-        <x:v>17</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J5" s="17" t="n">
-        <x:v>3490</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="K5" s="17" t="n">
         <x:f>IF(OR(I5="",J5=""),"",I5*J5)</x:f>
-        <x:v>59330</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="L5" s="17" t="n">
-        <x:v>4678</x:v>
+        <x:v>2139</x:v>
       </x:c>
       <x:c r="M5" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8241,7 +8249,7 @@
         <x:v>Permitted / described</x:v>
       </x:c>
       <x:c r="Q5" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="R5" s="14" t="str">
         <x:v>OCR pattern extraction</x:v>
@@ -8250,30 +8258,30 @@
         <x:v>OCR extracted - review recommended</x:v>
       </x:c>
       <x:c r="T5" s="13" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="U5" s="14" t="str">
-        <x:v>f emission unit (s) Eleven (11) 2,740 kw (3,673 engine HP) diesel-powered emergency generator sets; Seventeen (17) 3,490 kW (4,678 engine HP) diesel-powered emergency generator sets; and Twelve (12) cooling towers</x:v>
+        <x:v>Description of emission units to be operated: 1,500 KW (2,139 hp) Diesel Fueled Emergency Generator (Generator #7) Mail check and/or form to Illinols EPA, BOA-Permit Section, 1021 North Grand Ave. Ea</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="31.5" customHeight="1">
       <x:c r="A6" s="13" t="str">
-        <x:v>GEN-DOC-170001799908-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170001699320-AIR-002-01</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>IL_N_5</x:v>
+        <x:v>IL_N_23</x:v>
       </x:c>
       <x:c r="C6" s="15" t="str">
-        <x:v>170001799908</x:v>
+        <x:v>170001699320</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
-        <x:v>DOC-170001799908-AIR-001</x:v>
+        <x:v>DOC-170001699320-AIR-002</x:v>
       </x:c>
       <x:c r="E6" s="18" t="n">
-        <x:v>39924</x:v>
+        <x:v>40420</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
-        <x:v>CAAPP operating permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G6" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
@@ -8283,15 +8291,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J6" s="17" t="n">
-        <x:v>2500</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="K6" s="17" t="n">
         <x:f>IF(OR(I6="",J6=""),"",I6*J6)</x:f>
-        <x:v>7500</x:v>
-      </x:c>
-      <x:c r="L6" s="17" t="n">
-        <x:v>3750</x:v>
-      </x:c>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="L6" s="17"/>
       <x:c r="M6" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -8313,24 +8319,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U6" s="14" t="str">
-        <x:v>tee to CONSTRUCT and OPERATE emission unit (s) and/or air pollution control equipment consisting of three (3) 2,500 kW (3,750 HP) diesel emergency generator sets</x:v>
+        <x:v>ignated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of three 2,000 kW. (two (2) 2,876-HP and one (1) 3,937-HP) #2 fuel oil fired emergency generators</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="31.5" customHeight="1">
       <x:c r="A7" s="13" t="str">
-        <x:v>GEN-DOC-170002049806-AIR-002-01</x:v>
+        <x:v>GEN-DOC-170001764240-AIR-005-01</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>IL_N_6</x:v>
+        <x:v>IL_N_4</x:v>
       </x:c>
       <x:c r="C7" s="15" t="str">
-        <x:v>170002049806</x:v>
+        <x:v>170001764240</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>DOC-170002049806-AIR-002</x:v>
+        <x:v>DOC-170001764240-AIR-005</x:v>
       </x:c>
       <x:c r="E7" s="18" t="n">
-        <x:v>44336</x:v>
+        <x:v>44167</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8338,21 +8344,19 @@
       <x:c r="G7" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H7" s="14" t="str">
-        <x:v>EGEN1-EGEN4</x:v>
-      </x:c>
+      <x:c r="H7" s="14"/>
       <x:c r="I7" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="J7" s="17" t="n">
-        <x:v>1500</x:v>
+        <x:v>2740</x:v>
       </x:c>
       <x:c r="K7" s="17" t="n">
         <x:f>IF(OR(I7="",J7=""),"",I7*J7)</x:f>
-        <x:v>6000</x:v>
+        <x:v>30140</x:v>
       </x:c>
       <x:c r="L7" s="17" t="n">
-        <x:v>2012</x:v>
+        <x:v>3673</x:v>
       </x:c>
       <x:c r="M7" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8366,33 +8370,33 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R7" s="14" t="str">
-        <x:v>OCR + manual verification</x:v>
+        <x:v>OCR pattern extraction</x:v>
       </x:c>
       <x:c r="S7" s="14" t="str">
-        <x:v>Reviewed</x:v>
+        <x:v>OCR extracted - review recommended</x:v>
       </x:c>
       <x:c r="T7" s="13" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="U7" s="14" t="str">
-        <x:v>nted to the above-designated Permittee to OPERATE source (5) and/or air pollution control equipment consisting of: emission KW (2,012 engine HP) Diesel-Powered Emergency Generator Sets Four (4) 1,500 (EGEN1 - EGEN4) ; One (1) 2,000 . kW (2,682 engine HP) Dies...</x:v>
+        <x:v>ignated Permittee to OPERATE and/or air pollution control equipment consisting of emission unit (s) Eleven (11) 2,740 kw (3,673 engine HP) diesel-powered emergency generator sets; Seventeen (17) 3,490 kW (4,678 engine HP) diesel-powered emergency generator se...</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="31.5" customHeight="1">
       <x:c r="A8" s="13" t="str">
-        <x:v>GEN-DOC-170002049806-AIR-002-02</x:v>
+        <x:v>GEN-DOC-170001764240-AIR-005-02</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
-        <x:v>IL_N_6</x:v>
+        <x:v>IL_N_4</x:v>
       </x:c>
       <x:c r="C8" s="15" t="str">
-        <x:v>170002049806</x:v>
+        <x:v>170001764240</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
-        <x:v>DOC-170002049806-AIR-002</x:v>
+        <x:v>DOC-170001764240-AIR-005</x:v>
       </x:c>
       <x:c r="E8" s="18" t="n">
-        <x:v>44336</x:v>
+        <x:v>44167</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8400,21 +8404,19 @@
       <x:c r="G8" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H8" s="14" t="str">
-        <x:v>EGEN5</x:v>
-      </x:c>
+      <x:c r="H8" s="14"/>
       <x:c r="I8" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="J8" s="17" t="n">
-        <x:v>2000</x:v>
+        <x:v>3490</x:v>
       </x:c>
       <x:c r="K8" s="17" t="n">
         <x:f>IF(OR(I8="",J8=""),"",I8*J8)</x:f>
-        <x:v>2000</x:v>
+        <x:v>59330</x:v>
       </x:c>
       <x:c r="L8" s="17" t="n">
-        <x:v>2682</x:v>
+        <x:v>4678</x:v>
       </x:c>
       <x:c r="M8" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8428,53 +8430,53 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R8" s="14" t="str">
-        <x:v>OCR + manual verification</x:v>
+        <x:v>OCR pattern extraction</x:v>
       </x:c>
       <x:c r="S8" s="14" t="str">
-        <x:v>Reviewed</x:v>
+        <x:v>OCR extracted - review recommended</x:v>
       </x:c>
       <x:c r="T8" s="13" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="U8" s="14" t="str">
-        <x:v>trol equipment consisting of: emission KW (2,012 engine HP) Diesel-Powered Emergency Generator Sets Four (4) 1,500 (EGEN1 - EGEN4) ; One (1) 2,000 . kW (2,682 engine HP) Diesel-Powered Emergency Generator Set (EGEN 5) ; and</x:v>
+        <x:v>f emission unit (s) Eleven (11) 2,740 kw (3,673 engine HP) diesel-powered emergency generator sets; Seventeen (17) 3,490 kW (4,678 engine HP) diesel-powered emergency generator sets; and Twelve (12) cooling towers</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="31.5" customHeight="1">
       <x:c r="A9" s="13" t="str">
-        <x:v>GEN-DOC-170002290713-AIR-002-01</x:v>
+        <x:v>GEN-DOC-170001799908-AIR-001-01</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>IL_N_7</x:v>
+        <x:v>IL_N_5</x:v>
       </x:c>
       <x:c r="C9" s="15" t="str">
-        <x:v>170002290713</x:v>
+        <x:v>170001799908</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>DOC-170002290713-AIR-002</x:v>
+        <x:v>DOC-170001799908-AIR-001</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:v>44572</x:v>
+        <x:v>39924</x:v>
       </x:c>
       <x:c r="F9" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>CAAPP operating permit</x:v>
       </x:c>
       <x:c r="G9" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
+        <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H9" s="14"/>
       <x:c r="I9" s="17" t="n">
-        <x:v>22</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J9" s="17" t="n">
-        <x:v>3263</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="K9" s="17" t="n">
         <x:f>IF(OR(I9="",J9=""),"",I9*J9)</x:f>
-        <x:v>71786</x:v>
+        <x:v>7500</x:v>
       </x:c>
       <x:c r="L9" s="17" t="n">
-        <x:v>4376</x:v>
+        <x:v>3750</x:v>
       </x:c>
       <x:c r="M9" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8485,7 +8487,7 @@
         <x:v>Permitted / described</x:v>
       </x:c>
       <x:c r="Q9" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="R9" s="14" t="str">
         <x:v>OCR pattern extraction</x:v>
@@ -8497,24 +8499,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U9" s="14" t="str">
-        <x:v>rmittee to construct and/or air pollution control equipment consisting of twenty- emission unit (s) two (22) 4,376 BHP (3,263 KW) Diesel-Fired Emergency Generators (EG-01 - EG- : 22)</x:v>
+        <x:v>tee to CONSTRUCT and OPERATE emission unit (s) and/or air pollution control equipment consisting of three (3) 2,500 kW (3,750 HP) diesel emergency generator sets</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="31.5" customHeight="1">
       <x:c r="A10" s="13" t="str">
-        <x:v>GEN-DOC-170002394647-AIR-005-01</x:v>
+        <x:v>GEN-DOC-170002049806-AIR-002-01</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>IL_17</x:v>
+        <x:v>IL_N_6</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>170002394647</x:v>
+        <x:v>170002049806</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>DOC-170002394647-AIR-005</x:v>
+        <x:v>DOC-170002049806-AIR-002</x:v>
       </x:c>
       <x:c r="E10" s="18" t="n">
-        <x:v>44908</x:v>
+        <x:v>44336</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8522,19 +8524,21 @@
       <x:c r="G10" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H10" s="14"/>
+      <x:c r="H10" s="14" t="str">
+        <x:v>EGEN1-EGEN4</x:v>
+      </x:c>
       <x:c r="I10" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J10" s="17" t="n">
-        <x:v>2500</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="K10" s="17" t="n">
         <x:f>IF(OR(I10="",J10=""),"",I10*J10)</x:f>
-        <x:v>20000</x:v>
+        <x:v>6000</x:v>
       </x:c>
       <x:c r="L10" s="17" t="n">
-        <x:v>3599</x:v>
+        <x:v>2012</x:v>
       </x:c>
       <x:c r="M10" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8548,33 +8552,33 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R10" s="14" t="str">
-        <x:v>OCR pattern extraction</x:v>
+        <x:v>OCR + manual verification</x:v>
       </x:c>
       <x:c r="S10" s="14" t="str">
-        <x:v>OCR extracted - review recommended</x:v>
+        <x:v>Reviewed</x:v>
       </x:c>
       <x:c r="T10" s="13" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="U10" s="14" t="str">
-        <x:v>gnated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: Eight (8) 2,500 kW (3,599 HP) Diesel Emergency Generator Sets (Set C - Barn #3-#10); 1, Generators Six (6) 2,500 kw (3,680 HP) Diesel Emergency Generator Sets ...</x:v>
+        <x:v>nted to the above-designated Permittee to OPERATE source (5) and/or air pollution control equipment consisting of: emission KW (2,012 engine HP) Diesel-Powered Emergency Generator Sets Four (4) 1,500 (EGEN1 - EGEN4) ; One (1) 2,000 . kW (2,682 engine HP) Dies...</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="31.5" customHeight="1">
       <x:c r="A11" s="13" t="str">
-        <x:v>GEN-DOC-170002394647-AIR-005-02</x:v>
+        <x:v>GEN-DOC-170002049806-AIR-002-02</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
-        <x:v>IL_17</x:v>
+        <x:v>IL_N_6</x:v>
       </x:c>
       <x:c r="C11" s="15" t="str">
-        <x:v>170002394647</x:v>
+        <x:v>170002049806</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
-        <x:v>DOC-170002394647-AIR-005</x:v>
+        <x:v>DOC-170002049806-AIR-002</x:v>
       </x:c>
       <x:c r="E11" s="18" t="n">
-        <x:v>44908</x:v>
+        <x:v>44336</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8582,19 +8586,21 @@
       <x:c r="G11" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H11" s="14"/>
+      <x:c r="H11" s="14" t="str">
+        <x:v>EGEN5</x:v>
+      </x:c>
       <x:c r="I11" s="17" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="17" t="n">
-        <x:v>2500</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="K11" s="17" t="n">
         <x:f>IF(OR(I11="",J11=""),"",I11*J11)</x:f>
-        <x:v>15000</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="L11" s="17" t="n">
-        <x:v>3680</x:v>
+        <x:v>2682</x:v>
       </x:c>
       <x:c r="M11" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8608,53 +8614,53 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R11" s="14" t="str">
-        <x:v>OCR pattern extraction</x:v>
+        <x:v>OCR + manual verification</x:v>
       </x:c>
       <x:c r="S11" s="14" t="str">
-        <x:v>OCR extracted - review recommended</x:v>
+        <x:v>Reviewed</x:v>
       </x:c>
       <x:c r="T11" s="13" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="U11" s="14" t="str">
-        <x:v>Eight (8) 2,500 kW (3,599 HP) Diesel Emergency Generator Sets (Set C - Barn #3-#10); 1, Generators Six (6) 2,500 kw (3,680 HP) Diesel Emergency Generator Sets (Set A - Barn 2, Generators #24-#29); (8) 2,750 kW (4,060 engine HP) Diesel Emergency Generator Set</x:v>
+        <x:v>trol equipment consisting of: emission KW (2,012 engine HP) Diesel-Powered Emergency Generator Sets Four (4) 1,500 (EGEN1 - EGEN4) ; One (1) 2,000 . kW (2,682 engine HP) Diesel-Powered Emergency Generator Set (EGEN 5) ; and</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="31.5" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>GEN-DOC-170002394647-AIR-005-03</x:v>
+        <x:v>GEN-DOC-170002290713-AIR-002-01</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
-        <x:v>IL_17</x:v>
+        <x:v>IL_N_7</x:v>
       </x:c>
       <x:c r="C12" s="15" t="str">
-        <x:v>170002394647</x:v>
+        <x:v>170002290713</x:v>
       </x:c>
       <x:c r="D12" s="13" t="str">
-        <x:v>DOC-170002394647-AIR-005</x:v>
+        <x:v>DOC-170002290713-AIR-002</x:v>
       </x:c>
       <x:c r="E12" s="18" t="n">
-        <x:v>44908</x:v>
+        <x:v>44572</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>FESOP / operating permit</x:v>
+        <x:v>Construction permit</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
-        <x:v>Latest operating-permit inventory</x:v>
+        <x:v>Most recent permit with extractable inventory</x:v>
       </x:c>
       <x:c r="H12" s="14"/>
       <x:c r="I12" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="J12" s="17" t="n">
-        <x:v>2750</x:v>
+        <x:v>3263</x:v>
       </x:c>
       <x:c r="K12" s="17" t="n">
         <x:f>IF(OR(I12="",J12=""),"",I12*J12)</x:f>
-        <x:v>22000</x:v>
+        <x:v>71786</x:v>
       </x:c>
       <x:c r="L12" s="17" t="n">
-        <x:v>4060</x:v>
+        <x:v>4376</x:v>
       </x:c>
       <x:c r="M12" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8665,7 +8671,7 @@
         <x:v>Permitted / described</x:v>
       </x:c>
       <x:c r="Q12" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="R12" s="14" t="str">
         <x:v>OCR pattern extraction</x:v>
@@ -8677,12 +8683,12 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U12" s="14" t="str">
-        <x:v>s Six (6) 2,500 kw (3,680 HP) Diesel Emergency Generator Sets (Set A - Barn 2, Generators #24-#29); (8) 2,750 kW (4,060 engine HP) Diesel Emergency Generator Sets (Set B - Eight Four (4) 2,250 KW (3,353 HP) Diesel-powered Emergency Generator Sets (Set D); Iwe...</x:v>
+        <x:v>rmittee to construct and/or air pollution control equipment consisting of twenty- emission unit (s) two (22) 4,376 BHP (3,263 KW) Diesel-Fired Emergency Generators (EG-01 - EG- : 22)</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="31.5" customHeight="1">
       <x:c r="A13" s="13" t="str">
-        <x:v>GEN-DOC-170002394647-AIR-005-04</x:v>
+        <x:v>GEN-DOC-170002394647-AIR-005-01</x:v>
       </x:c>
       <x:c r="B13" s="13" t="str">
         <x:v>IL_17</x:v>
@@ -8704,17 +8710,17 @@
       </x:c>
       <x:c r="H13" s="14"/>
       <x:c r="I13" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J13" s="17" t="n">
-        <x:v>2250</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="K13" s="17" t="n">
         <x:f>IF(OR(I13="",J13=""),"",I13*J13)</x:f>
-        <x:v>9000</x:v>
+        <x:v>20000</x:v>
       </x:c>
       <x:c r="L13" s="17" t="n">
-        <x:v>3353</x:v>
+        <x:v>3599</x:v>
       </x:c>
       <x:c r="M13" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8737,12 +8743,12 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U13" s="14" t="str">
-        <x:v>Generators #24-#29); (8) 2,750 kW (4,060 engine HP) Diesel Emergency Generator Sets (Set B - Eight Four (4) 2,250 KW (3,353 HP) Diesel-powered Emergency Generator Sets (Set D); Iwenty-eight (28) 2,250 kW (3,223 HP). Diesel Emergency Generator Sets (A2-D2, Thi...</x:v>
+        <x:v>gnated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: Eight (8) 2,500 kW (3,599 HP) Diesel Emergency Generator Sets (Set C - Barn #3-#10); 1, Generators Six (6) 2,500 kw (3,680 HP) Diesel Emergency Generator Sets ...</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="31.5" customHeight="1">
       <x:c r="A14" s="13" t="str">
-        <x:v>GEN-DOC-170002394647-AIR-005-05</x:v>
+        <x:v>GEN-DOC-170002394647-AIR-005-02</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
         <x:v>IL_17</x:v>
@@ -8764,17 +8770,17 @@
       </x:c>
       <x:c r="H14" s="14"/>
       <x:c r="I14" s="17" t="n">
-        <x:v>28</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J14" s="17" t="n">
-        <x:v>2250</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="K14" s="17" t="n">
         <x:f>IF(OR(I14="",J14=""),"",I14*J14)</x:f>
-        <x:v>63000</x:v>
+        <x:v>15000</x:v>
       </x:c>
       <x:c r="L14" s="17" t="n">
-        <x:v>3223</x:v>
+        <x:v>3680</x:v>
       </x:c>
       <x:c r="M14" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8797,12 +8803,12 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U14" s="14" t="str">
-        <x:v>(Set B - Eight Four (4) 2,250 KW (3,353 HP) Diesel-powered Emergency Generator Sets (Set D); Iwenty-eight (28) 2,250 kW (3,223 HP). Diesel Emergency Generator Sets (A2-D2, Thirty-six (36) 2,250 kW (3,202 HP), Diesel-powered Generators (30A-30G, 30J 30R, 32A-3...</x:v>
+        <x:v>Eight (8) 2,500 kW (3,599 HP) Diesel Emergency Generator Sets (Set C - Barn #3-#10); 1, Generators Six (6) 2,500 kw (3,680 HP) Diesel Emergency Generator Sets (Set A - Barn 2, Generators #24-#29); (8) 2,750 kW (4,060 engine HP) Diesel Emergency Generator Set</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="31.5" customHeight="1">
       <x:c r="A15" s="13" t="str">
-        <x:v>GEN-DOC-170002394647-AIR-005-06</x:v>
+        <x:v>GEN-DOC-170002394647-AIR-005-03</x:v>
       </x:c>
       <x:c r="B15" s="13" t="str">
         <x:v>IL_17</x:v>
@@ -8824,17 +8830,17 @@
       </x:c>
       <x:c r="H15" s="14"/>
       <x:c r="I15" s="17" t="n">
-        <x:v>36</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J15" s="17" t="n">
-        <x:v>2250</x:v>
+        <x:v>2750</x:v>
       </x:c>
       <x:c r="K15" s="17" t="n">
         <x:f>IF(OR(I15="",J15=""),"",I15*J15)</x:f>
-        <x:v>81000</x:v>
+        <x:v>22000</x:v>
       </x:c>
       <x:c r="L15" s="17" t="n">
-        <x:v>3202</x:v>
+        <x:v>4060</x:v>
       </x:c>
       <x:c r="M15" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8857,24 +8863,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U15" s="14" t="str">
-        <x:v>Sets (Set D); Iwenty-eight (28) 2,250 kW (3,223 HP). Diesel Emergency Generator Sets (A2-D2, Thirty-six (36) 2,250 kW (3,202 HP), Diesel-powered Generators (30A-30G, 30J 30R, 32A-32G, 32J, 32R, 35A-35G, 35J, 35R, 37A-37G, 37J and 37R); One (1) 1,250kw (1</x:v>
+        <x:v>s Six (6) 2,500 kw (3,680 HP) Diesel Emergency Generator Sets (Set A - Barn 2, Generators #24-#29); (8) 2,750 kW (4,060 engine HP) Diesel Emergency Generator Sets (Set B - Eight Four (4) 2,250 KW (3,353 HP) Diesel-powered Emergency Generator Sets (Set D); Iwe...</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="31.5" customHeight="1">
       <x:c r="A16" s="13" t="str">
-        <x:v>GEN-DOC-170002399759-AIR-003-01</x:v>
+        <x:v>GEN-DOC-170002394647-AIR-005-04</x:v>
       </x:c>
       <x:c r="B16" s="13" t="str">
-        <x:v>IL_11</x:v>
+        <x:v>IL_17</x:v>
       </x:c>
       <x:c r="C16" s="15" t="str">
-        <x:v>170002399759</x:v>
+        <x:v>170002394647</x:v>
       </x:c>
       <x:c r="D16" s="13" t="str">
-        <x:v>DOC-170002399759-AIR-003</x:v>
+        <x:v>DOC-170002394647-AIR-005</x:v>
       </x:c>
       <x:c r="E16" s="18" t="n">
-        <x:v>45805</x:v>
+        <x:v>44908</x:v>
       </x:c>
       <x:c r="F16" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8884,17 +8890,17 @@
       </x:c>
       <x:c r="H16" s="14"/>
       <x:c r="I16" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J16" s="17" t="n">
-        <x:v>1000</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="K16" s="17" t="n">
         <x:f>IF(OR(I16="",J16=""),"",I16*J16)</x:f>
-        <x:v>1000</x:v>
+        <x:v>9000</x:v>
       </x:c>
       <x:c r="L16" s="17" t="n">
-        <x:v>1482</x:v>
+        <x:v>3353</x:v>
       </x:c>
       <x:c r="M16" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8917,24 +8923,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U16" s="14" t="str">
-        <x:v>gnated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: One (1)1000 kWe (1482 engine HP) Diesel-Powered Emergency Generator Sets (EG1) ; Twelve (12) 2,250 kWe (3,280 engine HP) Diesel-Powered Emergency Generator Set...</x:v>
+        <x:v>Generators #24-#29); (8) 2,750 kW (4,060 engine HP) Diesel Emergency Generator Sets (Set B - Eight Four (4) 2,250 KW (3,353 HP) Diesel-powered Emergency Generator Sets (Set D); Iwenty-eight (28) 2,250 kW (3,223 HP). Diesel Emergency Generator Sets (A2-D2, Thi...</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="31.5" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>GEN-DOC-170002399759-AIR-003-02</x:v>
+        <x:v>GEN-DOC-170002394647-AIR-005-05</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
-        <x:v>IL_11</x:v>
+        <x:v>IL_17</x:v>
       </x:c>
       <x:c r="C17" s="15" t="str">
-        <x:v>170002399759</x:v>
+        <x:v>170002394647</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>DOC-170002399759-AIR-003</x:v>
+        <x:v>DOC-170002394647-AIR-005</x:v>
       </x:c>
       <x:c r="E17" s="18" t="n">
-        <x:v>45805</x:v>
+        <x:v>44908</x:v>
       </x:c>
       <x:c r="F17" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -8944,17 +8950,17 @@
       </x:c>
       <x:c r="H17" s="14"/>
       <x:c r="I17" s="17" t="n">
-        <x:v>12</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="J17" s="17" t="n">
         <x:v>2250</x:v>
       </x:c>
       <x:c r="K17" s="17" t="n">
         <x:f>IF(OR(I17="",J17=""),"",I17*J17)</x:f>
-        <x:v>27000</x:v>
+        <x:v>63000</x:v>
       </x:c>
       <x:c r="L17" s="17" t="n">
-        <x:v>3280</x:v>
+        <x:v>3223</x:v>
       </x:c>
       <x:c r="M17" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -8977,24 +8983,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U17" s="14" t="str">
-        <x:v>ent consisting of: One (1)1000 kWe (1482 engine HP) Diesel-Powered Emergency Generator Sets (EG1) ; Twelve (12) 2,250 kWe (3,280 engine HP) Diesel-Powered Emergency Generator Sets (EG2-EG13); and Five (5) 2,500 kwe (3,640 engine HP) Diesel-Powered Emergency G...</x:v>
+        <x:v>(Set B - Eight Four (4) 2,250 KW (3,353 HP) Diesel-powered Emergency Generator Sets (Set D); Iwenty-eight (28) 2,250 kW (3,223 HP). Diesel Emergency Generator Sets (A2-D2, Thirty-six (36) 2,250 kW (3,202 HP), Diesel-powered Generators (30A-30G, 30J 30R, 32A-3...</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="31.5" customHeight="1">
       <x:c r="A18" s="13" t="str">
-        <x:v>GEN-DOC-170002399759-AIR-003-03</x:v>
+        <x:v>GEN-DOC-170002394647-AIR-005-06</x:v>
       </x:c>
       <x:c r="B18" s="13" t="str">
-        <x:v>IL_11</x:v>
+        <x:v>IL_17</x:v>
       </x:c>
       <x:c r="C18" s="15" t="str">
-        <x:v>170002399759</x:v>
+        <x:v>170002394647</x:v>
       </x:c>
       <x:c r="D18" s="13" t="str">
-        <x:v>DOC-170002399759-AIR-003</x:v>
+        <x:v>DOC-170002394647-AIR-005</x:v>
       </x:c>
       <x:c r="E18" s="18" t="n">
-        <x:v>45805</x:v>
+        <x:v>44908</x:v>
       </x:c>
       <x:c r="F18" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9004,17 +9010,17 @@
       </x:c>
       <x:c r="H18" s="14"/>
       <x:c r="I18" s="17" t="n">
-        <x:v>5</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="J18" s="17" t="n">
-        <x:v>2500</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="K18" s="17" t="n">
         <x:f>IF(OR(I18="",J18=""),"",I18*J18)</x:f>
-        <x:v>12500</x:v>
+        <x:v>81000</x:v>
       </x:c>
       <x:c r="L18" s="17" t="n">
-        <x:v>3640</x:v>
+        <x:v>3202</x:v>
       </x:c>
       <x:c r="M18" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -9037,24 +9043,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U18" s="14" t="str">
-        <x:v>) ; Twelve (12) 2,250 kWe (3,280 engine HP) Diesel-Powered Emergency Generator Sets (EG2-EG13); and Five (5) 2,500 kwe (3,640 engine HP) Diesel-Powered Emergency Generator Sets</x:v>
+        <x:v>Sets (Set D); Iwenty-eight (28) 2,250 kW (3,223 HP). Diesel Emergency Generator Sets (A2-D2, Thirty-six (36) 2,250 kW (3,202 HP), Diesel-powered Generators (30A-30G, 30J 30R, 32A-32G, 32J, 32R, 35A-35G, 35J, 35R, 37A-37G, 37J and 37R); One (1) 1,250kw (1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="31.5" customHeight="1">
       <x:c r="A19" s="13" t="str">
-        <x:v>GEN-DOC-170002406670-AIR-005-01</x:v>
+        <x:v>GEN-DOC-170002399759-AIR-003-01</x:v>
       </x:c>
       <x:c r="B19" s="13" t="str">
-        <x:v>IL_N_8</x:v>
+        <x:v>IL_11</x:v>
       </x:c>
       <x:c r="C19" s="15" t="str">
-        <x:v>170002406670</x:v>
+        <x:v>170002399759</x:v>
       </x:c>
       <x:c r="D19" s="13" t="str">
-        <x:v>DOC-170002406670-AIR-005</x:v>
+        <x:v>DOC-170002399759-AIR-003</x:v>
       </x:c>
       <x:c r="E19" s="18" t="n">
-        <x:v>46071</x:v>
+        <x:v>45805</x:v>
       </x:c>
       <x:c r="F19" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9064,16 +9070,18 @@
       </x:c>
       <x:c r="H19" s="14"/>
       <x:c r="I19" s="17" t="n">
-        <x:v>20</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="17" t="n">
-        <x:v>3250</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="K19" s="17" t="n">
         <x:f>IF(OR(I19="",J19=""),"",I19*J19)</x:f>
-        <x:v>65000</x:v>
-      </x:c>
-      <x:c r="L19" s="17"/>
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="L19" s="17" t="n">
+        <x:v>1482</x:v>
+      </x:c>
       <x:c r="M19" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9095,24 +9103,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U19" s="14" t="str">
-        <x:v>gnated Permittee to CONSTRUCT emission units) and/or air pollution control equipment consisting of: Twenty (20) 3,250 KW (4,701 BHP) Ultra-low Sulfur Diesel Emergency Generators (CH3-GEN201-A,B,C,D,E, CH3-GEN202-A,B,C,D,E, CH3-GEN301-A,B,C,D,E, CH3-GEN302-A,B...</x:v>
+        <x:v>gnated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: One (1)1000 kWe (1482 engine HP) Diesel-Powered Emergency Generator Sets (EG1) ; Twelve (12) 2,250 kWe (3,280 engine HP) Diesel-Powered Emergency Generator Set...</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="31.5" customHeight="1">
       <x:c r="A20" s="13" t="str">
-        <x:v>GEN-DOC-170002406670-AIR-005-02</x:v>
+        <x:v>GEN-DOC-170002399759-AIR-003-02</x:v>
       </x:c>
       <x:c r="B20" s="13" t="str">
-        <x:v>IL_N_8</x:v>
+        <x:v>IL_11</x:v>
       </x:c>
       <x:c r="C20" s="15" t="str">
-        <x:v>170002406670</x:v>
+        <x:v>170002399759</x:v>
       </x:c>
       <x:c r="D20" s="13" t="str">
-        <x:v>DOC-170002406670-AIR-005</x:v>
+        <x:v>DOC-170002399759-AIR-003</x:v>
       </x:c>
       <x:c r="E20" s="18" t="n">
-        <x:v>46071</x:v>
+        <x:v>45805</x:v>
       </x:c>
       <x:c r="F20" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9122,16 +9130,18 @@
       </x:c>
       <x:c r="H20" s="14"/>
       <x:c r="I20" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="J20" s="17" t="n">
-        <x:v>1500</x:v>
+        <x:v>2250</x:v>
       </x:c>
       <x:c r="K20" s="17" t="n">
         <x:f>IF(OR(I20="",J20=""),"",I20*J20)</x:f>
-        <x:v>1500</x:v>
-      </x:c>
-      <x:c r="L20" s="17"/>
+        <x:v>27000</x:v>
+      </x:c>
+      <x:c r="L20" s="17" t="n">
+        <x:v>3280</x:v>
+      </x:c>
       <x:c r="M20" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9153,24 +9163,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U20" s="14" t="str">
-        <x:v>enerators (CH3-GEN201-A,B,C,D,E, CH3-GEN202-A,B,C,D,E, CH3-GEN301-A,B,C,D,E, CH3-GEN302-A,B,C,D,E); One (1) 1,500 KW (2,220 BHP) Ultra-low Sulfur Diesel-Powered Emergency Generator (CH3-GEN-H01)</x:v>
+        <x:v>ent consisting of: One (1)1000 kWe (1482 engine HP) Diesel-Powered Emergency Generator Sets (EG1) ; Twelve (12) 2,250 kWe (3,280 engine HP) Diesel-Powered Emergency Generator Sets (EG2-EG13); and Five (5) 2,500 kwe (3,640 engine HP) Diesel-Powered Emergency G...</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="31.5" customHeight="1">
       <x:c r="A21" s="13" t="str">
-        <x:v>GEN-DOC-170002409427-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170002399759-AIR-003-03</x:v>
       </x:c>
       <x:c r="B21" s="13" t="str">
-        <x:v>IL_N_9</x:v>
+        <x:v>IL_11</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str">
-        <x:v>170002409427</x:v>
+        <x:v>170002399759</x:v>
       </x:c>
       <x:c r="D21" s="13" t="str">
-        <x:v>DOC-170002409427-AIR-001</x:v>
+        <x:v>DOC-170002399759-AIR-003</x:v>
       </x:c>
       <x:c r="E21" s="18" t="n">
-        <x:v>45490</x:v>
+        <x:v>45805</x:v>
       </x:c>
       <x:c r="F21" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9178,18 +9188,19 @@
       <x:c r="G21" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H21" s="14" t="str">
-        <x:v>Generator #1 - #2</x:v>
-      </x:c>
+      <x:c r="H21" s="14"/>
       <x:c r="I21" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J21" s="17"/>
-      <x:c r="K21" s="17" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J21" s="17" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="K21" s="17" t="n">
         <x:f>IF(OR(I21="",J21=""),"",I21*J21)</x:f>
+        <x:v>12500</x:v>
       </x:c>
       <x:c r="L21" s="17" t="n">
-        <x:v>2847</x:v>
+        <x:v>3640</x:v>
       </x:c>
       <x:c r="M21" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -9212,24 +9223,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U21" s="14" t="str">
-        <x:v>gnated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: Two (2) 2,847 hp Diesel-Powered Emergency Generator (Generator #1 - #2); 2,876 hp Diesel-Powered Emergency Generator (Generator #3); and one (1) One (1</x:v>
+        <x:v>) ; Twelve (12) 2,250 kWe (3,280 engine HP) Diesel-Powered Emergency Generator Sets (EG2-EG13); and Five (5) 2,500 kwe (3,640 engine HP) Diesel-Powered Emergency Generator Sets</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="31.5" customHeight="1">
       <x:c r="A22" s="13" t="str">
-        <x:v>GEN-DOC-170002409427-AIR-001-02</x:v>
+        <x:v>GEN-DOC-170002406670-AIR-005-01</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
-        <x:v>IL_N_9</x:v>
+        <x:v>IL_N_8</x:v>
       </x:c>
       <x:c r="C22" s="15" t="str">
-        <x:v>170002409427</x:v>
+        <x:v>170002406670</x:v>
       </x:c>
       <x:c r="D22" s="13" t="str">
-        <x:v>DOC-170002409427-AIR-001</x:v>
+        <x:v>DOC-170002406670-AIR-005</x:v>
       </x:c>
       <x:c r="E22" s="18" t="n">
-        <x:v>45490</x:v>
+        <x:v>46071</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9237,19 +9248,18 @@
       <x:c r="G22" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H22" s="14" t="str">
-        <x:v>Generator #4</x:v>
-      </x:c>
+      <x:c r="H22" s="14"/>
       <x:c r="I22" s="17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J22" s="17"/>
-      <x:c r="K22" s="17" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J22" s="17" t="n">
+        <x:v>3250</x:v>
+      </x:c>
+      <x:c r="K22" s="17" t="n">
         <x:f>IF(OR(I22="",J22=""),"",I22*J22)</x:f>
-      </x:c>
-      <x:c r="L22" s="17" t="n">
-        <x:v>1821</x:v>
-      </x:c>
+        <x:v>65000</x:v>
+      </x:c>
+      <x:c r="L22" s="17"/>
       <x:c r="M22" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9271,42 +9281,43 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U22" s="14" t="str">
-        <x:v>ency Generator (Generator #1 - #2); 2,876 hp Diesel-Powered Emergency Generator (Generator #3); and one (1) One (1) 1821 hp Diesel-Powered Emergency Generator (Generator #4)</x:v>
+        <x:v>gnated Permittee to CONSTRUCT emission units) and/or air pollution control equipment consisting of: Twenty (20) 3,250 KW (4,701 BHP) Ultra-low Sulfur Diesel Emergency Generators (CH3-GEN201-A,B,C,D,E, CH3-GEN202-A,B,C,D,E, CH3-GEN301-A,B,C,D,E, CH3-GEN302-A,B...</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
       <x:c r="A23" s="13" t="str">
-        <x:v>GEN-DOC-170002414983-AIR-004-01</x:v>
+        <x:v>GEN-DOC-170002406670-AIR-005-02</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>IL_N_22</x:v>
+        <x:v>IL_N_8</x:v>
       </x:c>
       <x:c r="C23" s="15" t="str">
-        <x:v>170002414983</x:v>
+        <x:v>170002406670</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
-        <x:v>DOC-170002414983-AIR-004</x:v>
+        <x:v>DOC-170002406670-AIR-005</x:v>
       </x:c>
       <x:c r="E23" s="18" t="n">
-        <x:v>45574</x:v>
+        <x:v>46071</x:v>
       </x:c>
       <x:c r="F23" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G23" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
+        <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H23" s="14"/>
       <x:c r="I23" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J23" s="17"/>
-      <x:c r="K23" s="17" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J23" s="17" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="K23" s="17" t="n">
         <x:f>IF(OR(I23="",J23=""),"",I23*J23)</x:f>
-      </x:c>
-      <x:c r="L23" s="17" t="n">
-        <x:v>4423</x:v>
-      </x:c>
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="L23" s="17"/>
       <x:c r="M23" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9328,24 +9339,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U23" s="14" t="str">
-        <x:v>nated Permittee to CONSTRUCT emission unit (s) and/or air pollution control equipment consisting of two (2) 4,423 HP Diesel-powered Emergency Generator Sets (1EY1.EG.01 and 2EY1. EG.01)</x:v>
+        <x:v>enerators (CH3-GEN201-A,B,C,D,E, CH3-GEN202-A,B,C,D,E, CH3-GEN301-A,B,C,D,E, CH3-GEN302-A,B,C,D,E); One (1) 1,500 KW (2,220 BHP) Ultra-low Sulfur Diesel-Powered Emergency Generator (CH3-GEN-H01)</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
       <x:c r="A24" s="13" t="str">
-        <x:v>GEN-DOC-170002425089-AIR-003-01</x:v>
+        <x:v>GEN-DOC-170002409427-AIR-001-01</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
-        <x:v>IL_13</x:v>
+        <x:v>IL_N_9</x:v>
       </x:c>
       <x:c r="C24" s="15" t="str">
-        <x:v>170002425089</x:v>
+        <x:v>170002409427</x:v>
       </x:c>
       <x:c r="D24" s="13" t="str">
-        <x:v>DOC-170002425089-AIR-003</x:v>
+        <x:v>DOC-170002409427-AIR-001</x:v>
       </x:c>
       <x:c r="E24" s="18" t="n">
-        <x:v>46030</x:v>
+        <x:v>45490</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9353,19 +9364,18 @@
       <x:c r="G24" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H24" s="14"/>
+      <x:c r="H24" s="14" t="str">
+        <x:v>Generator #1 - #2</x:v>
+      </x:c>
       <x:c r="I24" s="17" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="J24" s="17" t="n">
-        <x:v>3250</x:v>
-      </x:c>
-      <x:c r="K24" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J24" s="17"/>
+      <x:c r="K24" s="17" t="str">
         <x:f>IF(OR(I24="",J24=""),"",I24*J24)</x:f>
-        <x:v>48750</x:v>
       </x:c>
       <x:c r="L24" s="17" t="n">
-        <x:v>4680</x:v>
+        <x:v>2847</x:v>
       </x:c>
       <x:c r="M24" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
@@ -9388,24 +9398,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U24" s="14" t="str">
-        <x:v>signated Permittee to OPERATE emission units) and/or air pollution control equipment consisting of: Fifteen (15) 3,250 kWe (4,680 engine hp) Diesel-Powered Emergency Generator Sets (GEN01 - GEN15)</x:v>
+        <x:v>gnated Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: Two (2) 2,847 hp Diesel-Powered Emergency Generator (Generator #1 - #2); 2,876 hp Diesel-Powered Emergency Generator (Generator #3); and one (1) One (1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">
       <x:c r="A25" s="13" t="str">
-        <x:v>GEN-DOC-170002444709-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170002409427-AIR-001-02</x:v>
       </x:c>
       <x:c r="B25" s="13" t="str">
-        <x:v>IL_N_10</x:v>
+        <x:v>IL_N_9</x:v>
       </x:c>
       <x:c r="C25" s="15" t="str">
-        <x:v>170002444709</x:v>
+        <x:v>170002409427</x:v>
       </x:c>
       <x:c r="D25" s="13" t="str">
-        <x:v>DOC-170002444709-AIR-001</x:v>
+        <x:v>DOC-170002409427-AIR-001</x:v>
       </x:c>
       <x:c r="E25" s="18" t="n">
-        <x:v>46127</x:v>
+        <x:v>45490</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -9413,18 +9423,19 @@
       <x:c r="G25" s="14" t="str">
         <x:v>Latest operating-permit inventory</x:v>
       </x:c>
-      <x:c r="H25" s="14"/>
+      <x:c r="H25" s="14" t="str">
+        <x:v>Generator #4</x:v>
+      </x:c>
       <x:c r="I25" s="17" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J25" s="17" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="K25" s="17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J25" s="17"/>
+      <x:c r="K25" s="17" t="str">
         <x:f>IF(OR(I25="",J25=""),"",I25*J25)</x:f>
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="L25" s="17"/>
+      </x:c>
+      <x:c r="L25" s="17" t="n">
+        <x:v>1821</x:v>
+      </x:c>
       <x:c r="M25" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9446,43 +9457,42 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U25" s="14" t="str">
-        <x:v>signated Permittee to OPERATE emission units) and/or air pollution control equipment consisting of: Two (2) 500 KWe (762 hp engine) Diesel-Powered Emergency Generator Set (EG-101 and EG-121); and Thirty-two (32) 3, 100 KWe (4,376 hp engine) Diesel-Powered Eme...</x:v>
+        <x:v>ency Generator (Generator #1 - #2); 2,876 hp Diesel-Powered Emergency Generator (Generator #3); and one (1) One (1) 1821 hp Diesel-Powered Emergency Generator (Generator #4)</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="31.5" customHeight="1">
       <x:c r="A26" s="13" t="str">
-        <x:v>GEN-DOC-170002444709-AIR-001-02</x:v>
+        <x:v>GEN-DOC-170002414983-AIR-004-01</x:v>
       </x:c>
       <x:c r="B26" s="13" t="str">
-        <x:v>IL_N_10</x:v>
+        <x:v>IL_N_22</x:v>
       </x:c>
       <x:c r="C26" s="15" t="str">
-        <x:v>170002444709</x:v>
+        <x:v>170002414983</x:v>
       </x:c>
       <x:c r="D26" s="13" t="str">
-        <x:v>DOC-170002444709-AIR-001</x:v>
+        <x:v>DOC-170002414983-AIR-004</x:v>
       </x:c>
       <x:c r="E26" s="18" t="n">
-        <x:v>46127</x:v>
+        <x:v>45574</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>FESOP / operating permit</x:v>
+        <x:v>Construction permit</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>Latest operating-permit inventory</x:v>
+        <x:v>Most recent permit with extractable inventory</x:v>
       </x:c>
       <x:c r="H26" s="14"/>
       <x:c r="I26" s="17" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="J26" s="17" t="n">
-        <x:v>3100</x:v>
-      </x:c>
-      <x:c r="K26" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J26" s="17"/>
+      <x:c r="K26" s="17" t="str">
         <x:f>IF(OR(I26="",J26=""),"",I26*J26)</x:f>
-        <x:v>99200</x:v>
-      </x:c>
-      <x:c r="L26" s="17"/>
+      </x:c>
+      <x:c r="L26" s="17" t="n">
+        <x:v>4423</x:v>
+      </x:c>
       <x:c r="M26" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9504,43 +9514,45 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U26" s="14" t="str">
-        <x:v>of: Two (2) 500 KWe (762 hp engine) Diesel-Powered Emergency Generator Set (EG-101 and EG-121); and Thirty-two (32) 3, 100 KWe (4,376 hp engine) Diesel-Powered Emergency Generator Sets (EG-001- EG-032), as described in the above-referenced application</x:v>
+        <x:v>nated Permittee to CONSTRUCT emission unit (s) and/or air pollution control equipment consisting of two (2) 4,423 HP Diesel-powered Emergency Generator Sets (1EY1.EG.01 and 2EY1. EG.01)</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="31.5" customHeight="1">
       <x:c r="A27" s="13" t="str">
-        <x:v>GEN-DOC-170002468817-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170002425089-AIR-003-01</x:v>
       </x:c>
       <x:c r="B27" s="13" t="str">
-        <x:v>IL_22; IL_23</x:v>
+        <x:v>IL_13</x:v>
       </x:c>
       <x:c r="C27" s="15" t="str">
-        <x:v>170002468817</x:v>
+        <x:v>170002425089</x:v>
       </x:c>
       <x:c r="D27" s="13" t="str">
-        <x:v>DOC-170002468817-AIR-001</x:v>
+        <x:v>DOC-170002425089-AIR-003</x:v>
       </x:c>
       <x:c r="E27" s="18" t="n">
-        <x:v>44473</x:v>
+        <x:v>46030</x:v>
       </x:c>
       <x:c r="F27" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G27" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
+        <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H27" s="14"/>
       <x:c r="I27" s="17" t="n">
-        <x:v>49</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J27" s="17" t="n">
-        <x:v>3000</x:v>
+        <x:v>3250</x:v>
       </x:c>
       <x:c r="K27" s="17" t="n">
         <x:f>IF(OR(I27="",J27=""),"",I27*J27)</x:f>
-        <x:v>147000</x:v>
-      </x:c>
-      <x:c r="L27" s="17"/>
+        <x:v>48750</x:v>
+      </x:c>
+      <x:c r="L27" s="17" t="n">
+        <x:v>4680</x:v>
+      </x:c>
       <x:c r="M27" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9562,30 +9574,30 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U27" s="14" t="str">
-        <x:v>CONSTRUCT permit This emission unit(s) and/or air pollution control equipment consisting of: Forty-Nine (49) 3,000 KW (4,393 BHP) Diesel Emergency Generators; Two (2) 500 kw (762 BHP) Diesel Emergency Generators</x:v>
+        <x:v>signated Permittee to OPERATE emission units) and/or air pollution control equipment consisting of: Fifteen (15) 3,250 kWe (4,680 engine hp) Diesel-Powered Emergency Generator Sets (GEN01 - GEN15)</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="31.5" customHeight="1">
       <x:c r="A28" s="13" t="str">
-        <x:v>GEN-DOC-170002468817-AIR-001-02</x:v>
+        <x:v>GEN-DOC-170002444709-AIR-001-01</x:v>
       </x:c>
       <x:c r="B28" s="13" t="str">
-        <x:v>IL_22; IL_23</x:v>
+        <x:v>IL_N_10</x:v>
       </x:c>
       <x:c r="C28" s="15" t="str">
-        <x:v>170002468817</x:v>
+        <x:v>170002444709</x:v>
       </x:c>
       <x:c r="D28" s="13" t="str">
-        <x:v>DOC-170002468817-AIR-001</x:v>
+        <x:v>DOC-170002444709-AIR-001</x:v>
       </x:c>
       <x:c r="E28" s="18" t="n">
-        <x:v>44473</x:v>
+        <x:v>46127</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
+        <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H28" s="14"/>
       <x:c r="I28" s="17" t="n">
@@ -9620,41 +9632,41 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U28" s="14" t="str">
-        <x:v>control equipment consisting of: Forty-Nine (49) 3,000 KW (4,393 BHP) Diesel Emergency Generators; Two (2) 500 kw (762 BHP) Diesel Emergency Generators</x:v>
+        <x:v>signated Permittee to OPERATE emission units) and/or air pollution control equipment consisting of: Two (2) 500 KWe (762 hp engine) Diesel-Powered Emergency Generator Set (EG-101 and EG-121); and Thirty-two (32) 3, 100 KWe (4,376 hp engine) Diesel-Powered Eme...</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="31.5" customHeight="1">
       <x:c r="A29" s="13" t="str">
-        <x:v>GEN-DOC-170002484176-AIR-004-01</x:v>
+        <x:v>GEN-DOC-170002444709-AIR-001-02</x:v>
       </x:c>
       <x:c r="B29" s="13" t="str">
-        <x:v>IL_N_11</x:v>
+        <x:v>IL_N_10</x:v>
       </x:c>
       <x:c r="C29" s="15" t="str">
-        <x:v>170002484176</x:v>
+        <x:v>170002444709</x:v>
       </x:c>
       <x:c r="D29" s="13" t="str">
-        <x:v>DOC-170002484176-AIR-004</x:v>
+        <x:v>DOC-170002444709-AIR-001</x:v>
       </x:c>
       <x:c r="E29" s="18" t="n">
-        <x:v>45392</x:v>
+        <x:v>46127</x:v>
       </x:c>
       <x:c r="F29" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G29" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
+        <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H29" s="14"/>
       <x:c r="I29" s="17" t="n">
-        <x:v>18</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="J29" s="17" t="n">
-        <x:v>3000</x:v>
+        <x:v>3100</x:v>
       </x:c>
       <x:c r="K29" s="17" t="n">
         <x:f>IF(OR(I29="",J29=""),"",I29*J29)</x:f>
-        <x:v>54000</x:v>
+        <x:v>99200</x:v>
       </x:c>
       <x:c r="L29" s="17"/>
       <x:c r="M29" s="14" t="str">
@@ -9678,24 +9690,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U29" s="14" t="str">
-        <x:v>ated Permittee to CONSTRUCT emission unit (s) and/or air pollution control equipment consisting of: Eighteen (18) 3,000 kWe (4,680 HP, 4,423 HP, or 4,309 HP Engine) Diesel- Powered Emergency Generators (EG01 - EG18) (24) 1,500 kwe or 1,000 kwe (1,667 Kwm or 1...</x:v>
+        <x:v>of: Two (2) 500 KWe (762 hp engine) Diesel-Powered Emergency Generator Set (EG-101 and EG-121); and Thirty-two (32) 3, 100 KWe (4,376 hp engine) Diesel-Powered Emergency Generator Sets (EG-001- EG-032), as described in the above-referenced application</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="31.5" customHeight="1">
       <x:c r="A30" s="13" t="str">
-        <x:v>GEN-DOC-170002484176-AIR-004-02</x:v>
+        <x:v>GEN-DOC-170002468817-AIR-001-01</x:v>
       </x:c>
       <x:c r="B30" s="13" t="str">
-        <x:v>IL_N_11</x:v>
+        <x:v>IL_22; IL_23</x:v>
       </x:c>
       <x:c r="C30" s="15" t="str">
-        <x:v>170002484176</x:v>
+        <x:v>170002468817</x:v>
       </x:c>
       <x:c r="D30" s="13" t="str">
-        <x:v>DOC-170002484176-AIR-004</x:v>
+        <x:v>DOC-170002468817-AIR-001</x:v>
       </x:c>
       <x:c r="E30" s="18" t="n">
-        <x:v>45392</x:v>
+        <x:v>44473</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
         <x:v>Construction permit</x:v>
@@ -9705,14 +9717,14 @@
       </x:c>
       <x:c r="H30" s="14"/>
       <x:c r="I30" s="17" t="n">
-        <x:v>24</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="J30" s="17" t="n">
-        <x:v>1500</x:v>
+        <x:v>3000</x:v>
       </x:c>
       <x:c r="K30" s="17" t="n">
         <x:f>IF(OR(I30="",J30=""),"",I30*J30)</x:f>
-        <x:v>36000</x:v>
+        <x:v>147000</x:v>
       </x:c>
       <x:c r="L30" s="17"/>
       <x:c r="M30" s="14" t="str">
@@ -9736,24 +9748,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U30" s="14" t="str">
-        <x:v>000 kWe (4,680 HP, 4,423 HP, or 4,309 HP Engine) Diesel- Powered Emergency Generators (EG01 - EG18) (24) 1,500 kwe or 1,000 kwe (1,667 Kwm or 1,111 kWm Engine) Twenty four Diesel-Powered Emergency Generators (TEG01 - TEG24)</x:v>
+        <x:v>CONSTRUCT permit This emission unit(s) and/or air pollution control equipment consisting of: Forty-Nine (49) 3,000 KW (4,393 BHP) Diesel Emergency Generators; Two (2) 500 kw (762 BHP) Diesel Emergency Generators</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="31.5" customHeight="1">
       <x:c r="A31" s="13" t="str">
-        <x:v>GEN-DOC-170002499384-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170002468817-AIR-001-02</x:v>
       </x:c>
       <x:c r="B31" s="13" t="str">
-        <x:v>IL_N_13</x:v>
+        <x:v>IL_22; IL_23</x:v>
       </x:c>
       <x:c r="C31" s="15" t="str">
-        <x:v>170002499384</x:v>
+        <x:v>170002468817</x:v>
       </x:c>
       <x:c r="D31" s="13" t="str">
-        <x:v>DOC-170002499384-AIR-001</x:v>
+        <x:v>DOC-170002468817-AIR-001</x:v>
       </x:c>
       <x:c r="E31" s="18" t="n">
-        <x:v>44629</x:v>
+        <x:v>44473</x:v>
       </x:c>
       <x:c r="F31" s="14" t="str">
         <x:v>Construction permit</x:v>
@@ -9763,18 +9775,16 @@
       </x:c>
       <x:c r="H31" s="14"/>
       <x:c r="I31" s="17" t="n">
-        <x:v>20</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J31" s="17" t="n">
-        <x:v>3263</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="K31" s="17" t="n">
         <x:f>IF(OR(I31="",J31=""),"",I31*J31)</x:f>
-        <x:v>65260</x:v>
-      </x:c>
-      <x:c r="L31" s="17" t="n">
-        <x:v>4376</x:v>
-      </x:c>
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="L31" s="17"/>
       <x:c r="M31" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9796,24 +9806,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U31" s="14" t="str">
-        <x:v>ttee to construct This permit emission unit(s) and/or air pollution control equipment consisting of twenty (20) 4,376 BHP (3,263 KW) Diesel-Fired Emergency Generators (EG-02 - EG-21) one (1) 762 BHP (569 kW) Diesel-Fired Emergency Generator (EG-01) and</x:v>
+        <x:v>control equipment consisting of: Forty-Nine (49) 3,000 KW (4,393 BHP) Diesel Emergency Generators; Two (2) 500 kw (762 BHP) Diesel Emergency Generators</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="31.5" customHeight="1">
       <x:c r="A32" s="13" t="str">
-        <x:v>GEN-DOC-170002499384-AIR-001-02</x:v>
+        <x:v>GEN-DOC-170002484176-AIR-004-01</x:v>
       </x:c>
       <x:c r="B32" s="13" t="str">
-        <x:v>IL_N_13</x:v>
+        <x:v>IL_N_11</x:v>
       </x:c>
       <x:c r="C32" s="15" t="str">
-        <x:v>170002499384</x:v>
+        <x:v>170002484176</x:v>
       </x:c>
       <x:c r="D32" s="13" t="str">
-        <x:v>DOC-170002499384-AIR-001</x:v>
+        <x:v>DOC-170002484176-AIR-004</x:v>
       </x:c>
       <x:c r="E32" s="18" t="n">
-        <x:v>44629</x:v>
+        <x:v>45392</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>Construction permit</x:v>
@@ -9823,18 +9833,16 @@
       </x:c>
       <x:c r="H32" s="14"/>
       <x:c r="I32" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="J32" s="17" t="n">
-        <x:v>569</x:v>
+        <x:v>3000</x:v>
       </x:c>
       <x:c r="K32" s="17" t="n">
         <x:f>IF(OR(I32="",J32=""),"",I32*J32)</x:f>
-        <x:v>569</x:v>
-      </x:c>
-      <x:c r="L32" s="17" t="n">
-        <x:v>762</x:v>
-      </x:c>
+        <x:v>54000</x:v>
+      </x:c>
+      <x:c r="L32" s="17"/>
       <x:c r="M32" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9856,45 +9864,43 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U32" s="14" t="str">
-        <x:v>nt consisting of twenty (20) 4,376 BHP (3,263 KW) Diesel-Fired Emergency Generators (EG-02 - EG-21) one (1) 762 BHP (569 kW) Diesel-Fired Emergency Generator (EG-01) and</x:v>
+        <x:v>ated Permittee to CONSTRUCT emission unit (s) and/or air pollution control equipment consisting of: Eighteen (18) 3,000 kWe (4,680 HP, 4,423 HP, or 4,309 HP Engine) Diesel- Powered Emergency Generators (EG01 - EG18) (24) 1,500 kwe or 1,000 kwe (1,667 Kwm or 1...</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="31.5" customHeight="1">
       <x:c r="A33" s="13" t="str">
-        <x:v>GEN-DOC-170002516267-AIR-004-01</x:v>
+        <x:v>GEN-DOC-170002484176-AIR-004-02</x:v>
       </x:c>
       <x:c r="B33" s="13" t="str">
-        <x:v>IL_12</x:v>
+        <x:v>IL_N_11</x:v>
       </x:c>
       <x:c r="C33" s="15" t="str">
-        <x:v>170002516267</x:v>
+        <x:v>170002484176</x:v>
       </x:c>
       <x:c r="D33" s="13" t="str">
-        <x:v>DOC-170002516267-AIR-004</x:v>
+        <x:v>DOC-170002484176-AIR-004</x:v>
       </x:c>
       <x:c r="E33" s="18" t="n">
-        <x:v>45419</x:v>
+        <x:v>45392</x:v>
       </x:c>
       <x:c r="F33" s="14" t="str">
-        <x:v>FESOP / operating permit</x:v>
+        <x:v>Construction permit</x:v>
       </x:c>
       <x:c r="G33" s="14" t="str">
-        <x:v>Latest operating-permit inventory</x:v>
+        <x:v>Most recent permit with extractable inventory</x:v>
       </x:c>
       <x:c r="H33" s="14"/>
       <x:c r="I33" s="17" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="J33" s="17" t="n">
-        <x:v>2500</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="K33" s="17" t="n">
         <x:f>IF(OR(I33="",J33=""),"",I33*J33)</x:f>
-        <x:v>62500</x:v>
-      </x:c>
-      <x:c r="L33" s="17" t="n">
-        <x:v>3640</x:v>
-      </x:c>
+        <x:v>36000</x:v>
+      </x:c>
+      <x:c r="L33" s="17"/>
       <x:c r="M33" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
@@ -9916,50 +9922,50 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U33" s="14" t="str">
-        <x:v>Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: Iwenty-five (25) 2,500 kwe (3,640 engine HP) Diesel-Powered Emergency Generator Sets (GEN-P1 - GEN-P16, GEN-M1 - GEN-M6 and GEN-RI - GEN-R3)</x:v>
+        <x:v>000 kWe (4,680 HP, 4,423 HP, or 4,309 HP Engine) Diesel- Powered Emergency Generators (EG01 - EG18) (24) 1,500 kwe or 1,000 kwe (1,667 Kwm or 1,111 kWm Engine) Twenty four Diesel-Powered Emergency Generators (TEG01 - TEG24)</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="31.5" customHeight="1">
       <x:c r="A34" s="13" t="str">
-        <x:v>GEN-DOC-170002600200-AIR-003-01</x:v>
+        <x:v>GEN-DOC-170002499384-AIR-001-01</x:v>
       </x:c>
       <x:c r="B34" s="13" t="str">
-        <x:v>IL_N_18</x:v>
+        <x:v>IL_N_13</x:v>
       </x:c>
       <x:c r="C34" s="15" t="str">
-        <x:v>170002600200</x:v>
+        <x:v>170002499384</x:v>
       </x:c>
       <x:c r="D34" s="13" t="str">
-        <x:v>DOC-170002600200-AIR-003</x:v>
+        <x:v>DOC-170002499384-AIR-001</x:v>
       </x:c>
       <x:c r="E34" s="18" t="n">
-        <x:v>46163</x:v>
+        <x:v>44629</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>FESOP / operating permit</x:v>
+        <x:v>Construction permit</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>Latest operating-permit inventory</x:v>
+        <x:v>Most recent permit with extractable inventory</x:v>
       </x:c>
       <x:c r="H34" s="14"/>
       <x:c r="I34" s="17" t="n">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="J34" s="17" t="n">
-        <x:v>3500</x:v>
+        <x:v>3263</x:v>
       </x:c>
       <x:c r="K34" s="17" t="n">
         <x:f>IF(OR(I34="",J34=""),"",I34*J34)</x:f>
-        <x:v>42000</x:v>
-      </x:c>
-      <x:c r="L34" s="17"/>
+        <x:v>65260</x:v>
+      </x:c>
+      <x:c r="L34" s="17" t="n">
+        <x:v>4376</x:v>
+      </x:c>
       <x:c r="M34" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
       <x:c r="N34" s="14"/>
-      <x:c r="O34" s="14" t="str">
-        <x:v>Diesel particulate filter</x:v>
-      </x:c>
+      <x:c r="O34" s="14"/>
       <x:c r="P34" s="14" t="str">
         <x:v>Permitted / described</x:v>
       </x:c>
@@ -9976,50 +9982,50 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U34" s="14" t="str">
-        <x:v>ignated Permittee to OPERATE emission unit(s) and/or air pollution control equipment consisting of: Twelve (12) 3,500 kW Diesel-Powered Emergency Generators Controlled by Diesel Particulate Filters; Two (2) 3,500 kW Diesel-Powered Emergency Generators; and</x:v>
+        <x:v>ttee to construct This permit emission unit(s) and/or air pollution control equipment consisting of twenty (20) 4,376 BHP (3,263 KW) Diesel-Fired Emergency Generators (EG-02 - EG-21) one (1) 762 BHP (569 kW) Diesel-Fired Emergency Generator (EG-01) and</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="31.5" customHeight="1">
       <x:c r="A35" s="13" t="str">
-        <x:v>GEN-DOC-170002600200-AIR-003-02</x:v>
+        <x:v>GEN-DOC-170002499384-AIR-001-02</x:v>
       </x:c>
       <x:c r="B35" s="13" t="str">
-        <x:v>IL_N_18</x:v>
+        <x:v>IL_N_13</x:v>
       </x:c>
       <x:c r="C35" s="15" t="str">
-        <x:v>170002600200</x:v>
+        <x:v>170002499384</x:v>
       </x:c>
       <x:c r="D35" s="13" t="str">
-        <x:v>DOC-170002600200-AIR-003</x:v>
+        <x:v>DOC-170002499384-AIR-001</x:v>
       </x:c>
       <x:c r="E35" s="18" t="n">
-        <x:v>46163</x:v>
+        <x:v>44629</x:v>
       </x:c>
       <x:c r="F35" s="14" t="str">
-        <x:v>FESOP / operating permit</x:v>
+        <x:v>Construction permit</x:v>
       </x:c>
       <x:c r="G35" s="14" t="str">
-        <x:v>Latest operating-permit inventory</x:v>
+        <x:v>Most recent permit with extractable inventory</x:v>
       </x:c>
       <x:c r="H35" s="14"/>
       <x:c r="I35" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J35" s="17" t="n">
-        <x:v>3500</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="K35" s="17" t="n">
         <x:f>IF(OR(I35="",J35=""),"",I35*J35)</x:f>
-        <x:v>7000</x:v>
-      </x:c>
-      <x:c r="L35" s="17"/>
+        <x:v>569</x:v>
+      </x:c>
+      <x:c r="L35" s="17" t="n">
+        <x:v>762</x:v>
+      </x:c>
       <x:c r="M35" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
       <x:c r="N35" s="14"/>
-      <x:c r="O35" s="14" t="str">
-        <x:v>Diesel particulate filter</x:v>
-      </x:c>
+      <x:c r="O35" s="14"/>
       <x:c r="P35" s="14" t="str">
         <x:v>Permitted / described</x:v>
       </x:c>
@@ -10036,24 +10042,24 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U35" s="14" t="str">
-        <x:v>Twelve (12) 3,500 kW Diesel-Powered Emergency Generators Controlled by Diesel Particulate Filters; Two (2) 3,500 kW Diesel-Powered Emergency Generators; and One (1) 800 KW Diesel-Powered Emergency Generator, as described in the above-referenced applic</x:v>
+        <x:v>nt consisting of twenty (20) 4,376 BHP (3,263 KW) Diesel-Fired Emergency Generators (EG-02 - EG-21) one (1) 762 BHP (569 kW) Diesel-Fired Emergency Generator (EG-01) and</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="31.5" customHeight="1">
       <x:c r="A36" s="13" t="str">
-        <x:v>GEN-DOC-170002600200-AIR-003-03</x:v>
+        <x:v>GEN-DOC-170002516267-AIR-004-01</x:v>
       </x:c>
       <x:c r="B36" s="13" t="str">
-        <x:v>IL_N_18</x:v>
+        <x:v>IL_12</x:v>
       </x:c>
       <x:c r="C36" s="15" t="str">
-        <x:v>170002600200</x:v>
+        <x:v>170002516267</x:v>
       </x:c>
       <x:c r="D36" s="13" t="str">
-        <x:v>DOC-170002600200-AIR-003</x:v>
+        <x:v>DOC-170002516267-AIR-004</x:v>
       </x:c>
       <x:c r="E36" s="18" t="n">
-        <x:v>46163</x:v>
+        <x:v>45419</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
         <x:v>FESOP / operating permit</x:v>
@@ -10063,23 +10069,23 @@
       </x:c>
       <x:c r="H36" s="14"/>
       <x:c r="I36" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="J36" s="17" t="n">
-        <x:v>800</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="K36" s="17" t="n">
         <x:f>IF(OR(I36="",J36=""),"",I36*J36)</x:f>
-        <x:v>800</x:v>
-      </x:c>
-      <x:c r="L36" s="17"/>
+        <x:v>62500</x:v>
+      </x:c>
+      <x:c r="L36" s="17" t="n">
+        <x:v>3640</x:v>
+      </x:c>
       <x:c r="M36" s="14" t="str">
         <x:v>Diesel / distillate fuel oil</x:v>
       </x:c>
       <x:c r="N36" s="14"/>
-      <x:c r="O36" s="14" t="str">
-        <x:v>Diesel particulate filter</x:v>
-      </x:c>
+      <x:c r="O36" s="14"/>
       <x:c r="P36" s="14" t="str">
         <x:v>Permitted / described</x:v>
       </x:c>
@@ -10096,43 +10102,41 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U36" s="14" t="str">
-        <x:v>Controlled by Diesel Particulate Filters; Two (2) 3,500 kW Diesel-Powered Emergency Generators; and One (1) 800 KW Diesel-Powered Emergency Generator, as described in the above-referenced application</x:v>
+        <x:v>Permittee to OPERATE emission unit (s) and/or air pollution control equipment consisting of: Iwenty-five (25) 2,500 kwe (3,640 engine HP) Diesel-Powered Emergency Generator Sets (GEN-P1 - GEN-P16, GEN-M1 - GEN-M6 and GEN-RI - GEN-R3)</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="31.5" customHeight="1">
       <x:c r="A37" s="13" t="str">
-        <x:v>GEN-DOC-170002620180-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170002600200-AIR-003-01</x:v>
       </x:c>
       <x:c r="B37" s="13" t="str">
-        <x:v>IL_1</x:v>
+        <x:v>IL_N_18</x:v>
       </x:c>
       <x:c r="C37" s="15" t="str">
-        <x:v>170002620180</x:v>
+        <x:v>170002600200</x:v>
       </x:c>
       <x:c r="D37" s="13" t="str">
-        <x:v>DOC-170002620180-AIR-001</x:v>
+        <x:v>DOC-170002600200-AIR-003</x:v>
       </x:c>
       <x:c r="E37" s="18" t="n">
-        <x:v>45461</x:v>
+        <x:v>46163</x:v>
       </x:c>
       <x:c r="F37" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G37" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
-      </x:c>
-      <x:c r="H37" s="14" t="str">
-        <x:v>G1-G64</x:v>
-      </x:c>
+        <x:v>Latest operating-permit inventory</x:v>
+      </x:c>
+      <x:c r="H37" s="14"/>
       <x:c r="I37" s="17" t="n">
-        <x:v>64</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="J37" s="17" t="n">
-        <x:v>685</x:v>
+        <x:v>3500</x:v>
       </x:c>
       <x:c r="K37" s="17" t="n">
         <x:f>IF(OR(I37="",J37=""),"",I37*J37)</x:f>
-        <x:v>43840</x:v>
+        <x:v>42000</x:v>
       </x:c>
       <x:c r="L37" s="17"/>
       <x:c r="M37" s="14" t="str">
@@ -10140,7 +10144,7 @@
       </x:c>
       <x:c r="N37" s="14"/>
       <x:c r="O37" s="14" t="str">
-        <x:v>Selective catalytic reduction</x:v>
+        <x:v>Diesel particulate filter</x:v>
       </x:c>
       <x:c r="P37" s="14" t="str">
         <x:v>Permitted / described</x:v>
@@ -10158,43 +10162,41 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U37" s="14" t="str">
-        <x:v>Permittee to CONSTRUCT This emission unit (s) and/or air pollution control equipment consisting of: Sixty-four (64) 685 kW (932 BHP) Diesel Non-Emergency Generators (G1-G64) equipped with Selective Catalytic Reduction (SCR) and Ammonia Slip Catalyst Control D...</x:v>
+        <x:v>ignated Permittee to OPERATE emission unit(s) and/or air pollution control equipment consisting of: Twelve (12) 3,500 kW Diesel-Powered Emergency Generators Controlled by Diesel Particulate Filters; Two (2) 3,500 kW Diesel-Powered Emergency Generators; and</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="31.5" customHeight="1">
       <x:c r="A38" s="13" t="str">
-        <x:v>GEN-DOC-170002620180-AIR-001-02</x:v>
+        <x:v>GEN-DOC-170002600200-AIR-003-02</x:v>
       </x:c>
       <x:c r="B38" s="13" t="str">
-        <x:v>IL_1</x:v>
+        <x:v>IL_N_18</x:v>
       </x:c>
       <x:c r="C38" s="15" t="str">
-        <x:v>170002620180</x:v>
+        <x:v>170002600200</x:v>
       </x:c>
       <x:c r="D38" s="13" t="str">
-        <x:v>DOC-170002620180-AIR-001</x:v>
+        <x:v>DOC-170002600200-AIR-003</x:v>
       </x:c>
       <x:c r="E38" s="18" t="n">
-        <x:v>45461</x:v>
+        <x:v>46163</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
-      </x:c>
-      <x:c r="H38" s="14" t="str">
-        <x:v>G65-G66</x:v>
-      </x:c>
+        <x:v>Latest operating-permit inventory</x:v>
+      </x:c>
+      <x:c r="H38" s="14"/>
       <x:c r="I38" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="J38" s="17" t="n">
-        <x:v>715</x:v>
+        <x:v>3500</x:v>
       </x:c>
       <x:c r="K38" s="17" t="n">
         <x:f>IF(OR(I38="",J38=""),"",I38*J38)</x:f>
-        <x:v>1430</x:v>
+        <x:v>7000</x:v>
       </x:c>
       <x:c r="L38" s="17"/>
       <x:c r="M38" s="14" t="str">
@@ -10202,7 +10204,7 @@
       </x:c>
       <x:c r="N38" s="14"/>
       <x:c r="O38" s="14" t="str">
-        <x:v>Selective catalytic reduction</x:v>
+        <x:v>Diesel particulate filter</x:v>
       </x:c>
       <x:c r="P38" s="14" t="str">
         <x:v>Permitted / described</x:v>
@@ -10220,41 +10222,41 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U38" s="14" t="str">
-        <x:v>quipped with Selective Catalytic Reduction (SCR) and Ammonia Slip Catalyst Control Devices; and Iwo (2) 715 kW (973 BHP) Diesel Emergency Generators (G65-G66)</x:v>
+        <x:v>Twelve (12) 3,500 kW Diesel-Powered Emergency Generators Controlled by Diesel Particulate Filters; Two (2) 3,500 kW Diesel-Powered Emergency Generators; and One (1) 800 KW Diesel-Powered Emergency Generator, as described in the above-referenced applic</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="31.5" customHeight="1">
       <x:c r="A39" s="13" t="str">
-        <x:v>GEN-DOC-170002671954-AIR-001-01</x:v>
+        <x:v>GEN-DOC-170002600200-AIR-003-03</x:v>
       </x:c>
       <x:c r="B39" s="13" t="str">
-        <x:v>IL_N_20</x:v>
+        <x:v>IL_N_18</x:v>
       </x:c>
       <x:c r="C39" s="15" t="str">
-        <x:v>170002671954</x:v>
+        <x:v>170002600200</x:v>
       </x:c>
       <x:c r="D39" s="13" t="str">
-        <x:v>DOC-170002671954-AIR-001</x:v>
+        <x:v>DOC-170002600200-AIR-003</x:v>
       </x:c>
       <x:c r="E39" s="18" t="n">
-        <x:v>45853</x:v>
+        <x:v>46163</x:v>
       </x:c>
       <x:c r="F39" s="14" t="str">
-        <x:v>Construction permit</x:v>
+        <x:v>FESOP / operating permit</x:v>
       </x:c>
       <x:c r="G39" s="14" t="str">
-        <x:v>Most recent permit with extractable inventory</x:v>
+        <x:v>Latest operating-permit inventory</x:v>
       </x:c>
       <x:c r="H39" s="14"/>
       <x:c r="I39" s="17" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J39" s="17" t="n">
-        <x:v>3250</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="K39" s="17" t="n">
         <x:f>IF(OR(I39="",J39=""),"",I39*J39)</x:f>
-        <x:v>126750</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="L39" s="17"/>
       <x:c r="M39" s="14" t="str">
@@ -10280,24 +10282,208 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="U39" s="14" t="str">
+        <x:v>Controlled by Diesel Particulate Filters; Two (2) 3,500 kW Diesel-Powered Emergency Generators; and One (1) 800 KW Diesel-Powered Emergency Generator, as described in the above-referenced application</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="31.5" customHeight="1">
+      <x:c r="A40" s="13" t="str">
+        <x:v>GEN-DOC-170002620180-AIR-001-01</x:v>
+      </x:c>
+      <x:c r="B40" s="13" t="str">
+        <x:v>IL_1</x:v>
+      </x:c>
+      <x:c r="C40" s="15" t="str">
+        <x:v>170002620180</x:v>
+      </x:c>
+      <x:c r="D40" s="13" t="str">
+        <x:v>DOC-170002620180-AIR-001</x:v>
+      </x:c>
+      <x:c r="E40" s="18" t="n">
+        <x:v>45461</x:v>
+      </x:c>
+      <x:c r="F40" s="14" t="str">
+        <x:v>Construction permit</x:v>
+      </x:c>
+      <x:c r="G40" s="14" t="str">
+        <x:v>Most recent permit with extractable inventory</x:v>
+      </x:c>
+      <x:c r="H40" s="14" t="str">
+        <x:v>G1-G64</x:v>
+      </x:c>
+      <x:c r="I40" s="17" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="J40" s="17" t="n">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="K40" s="17" t="n">
+        <x:f>IF(OR(I40="",J40=""),"",I40*J40)</x:f>
+        <x:v>43840</x:v>
+      </x:c>
+      <x:c r="L40" s="17"/>
+      <x:c r="M40" s="14" t="str">
+        <x:v>Diesel / distillate fuel oil</x:v>
+      </x:c>
+      <x:c r="N40" s="14"/>
+      <x:c r="O40" s="14" t="str">
+        <x:v>Selective catalytic reduction</x:v>
+      </x:c>
+      <x:c r="P40" s="14" t="str">
+        <x:v>Permitted / described</x:v>
+      </x:c>
+      <x:c r="Q40" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R40" s="14" t="str">
+        <x:v>OCR pattern extraction</x:v>
+      </x:c>
+      <x:c r="S40" s="14" t="str">
+        <x:v>OCR extracted - review recommended</x:v>
+      </x:c>
+      <x:c r="T40" s="13" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="U40" s="14" t="str">
+        <x:v>Permittee to CONSTRUCT This emission unit (s) and/or air pollution control equipment consisting of: Sixty-four (64) 685 kW (932 BHP) Diesel Non-Emergency Generators (G1-G64) equipped with Selective Catalytic Reduction (SCR) and Ammonia Slip Catalyst Control D...</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="31.5" customHeight="1">
+      <x:c r="A41" s="13" t="str">
+        <x:v>GEN-DOC-170002620180-AIR-001-02</x:v>
+      </x:c>
+      <x:c r="B41" s="13" t="str">
+        <x:v>IL_1</x:v>
+      </x:c>
+      <x:c r="C41" s="15" t="str">
+        <x:v>170002620180</x:v>
+      </x:c>
+      <x:c r="D41" s="13" t="str">
+        <x:v>DOC-170002620180-AIR-001</x:v>
+      </x:c>
+      <x:c r="E41" s="18" t="n">
+        <x:v>45461</x:v>
+      </x:c>
+      <x:c r="F41" s="14" t="str">
+        <x:v>Construction permit</x:v>
+      </x:c>
+      <x:c r="G41" s="14" t="str">
+        <x:v>Most recent permit with extractable inventory</x:v>
+      </x:c>
+      <x:c r="H41" s="14" t="str">
+        <x:v>G65-G66</x:v>
+      </x:c>
+      <x:c r="I41" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J41" s="17" t="n">
+        <x:v>715</x:v>
+      </x:c>
+      <x:c r="K41" s="17" t="n">
+        <x:f>IF(OR(I41="",J41=""),"",I41*J41)</x:f>
+        <x:v>1430</x:v>
+      </x:c>
+      <x:c r="L41" s="17"/>
+      <x:c r="M41" s="14" t="str">
+        <x:v>Diesel / distillate fuel oil</x:v>
+      </x:c>
+      <x:c r="N41" s="14"/>
+      <x:c r="O41" s="14" t="str">
+        <x:v>Selective catalytic reduction</x:v>
+      </x:c>
+      <x:c r="P41" s="14" t="str">
+        <x:v>Permitted / described</x:v>
+      </x:c>
+      <x:c r="Q41" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R41" s="14" t="str">
+        <x:v>OCR pattern extraction</x:v>
+      </x:c>
+      <x:c r="S41" s="14" t="str">
+        <x:v>OCR extracted - review recommended</x:v>
+      </x:c>
+      <x:c r="T41" s="13" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="U41" s="14" t="str">
+        <x:v>quipped with Selective Catalytic Reduction (SCR) and Ammonia Slip Catalyst Control Devices; and Iwo (2) 715 kW (973 BHP) Diesel Emergency Generators (G65-G66)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="31.5" customHeight="1">
+      <x:c r="A42" s="13" t="str">
+        <x:v>GEN-DOC-170002671954-AIR-001-01</x:v>
+      </x:c>
+      <x:c r="B42" s="13" t="str">
+        <x:v>IL_N_20</x:v>
+      </x:c>
+      <x:c r="C42" s="15" t="str">
+        <x:v>170002671954</x:v>
+      </x:c>
+      <x:c r="D42" s="13" t="str">
+        <x:v>DOC-170002671954-AIR-001</x:v>
+      </x:c>
+      <x:c r="E42" s="18" t="n">
+        <x:v>45853</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>Construction permit</x:v>
+      </x:c>
+      <x:c r="G42" s="14" t="str">
+        <x:v>Most recent permit with extractable inventory</x:v>
+      </x:c>
+      <x:c r="H42" s="14"/>
+      <x:c r="I42" s="17" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="J42" s="17" t="n">
+        <x:v>3250</x:v>
+      </x:c>
+      <x:c r="K42" s="17" t="n">
+        <x:f>IF(OR(I42="",J42=""),"",I42*J42)</x:f>
+        <x:v>126750</x:v>
+      </x:c>
+      <x:c r="L42" s="17"/>
+      <x:c r="M42" s="14" t="str">
+        <x:v>Diesel / distillate fuel oil</x:v>
+      </x:c>
+      <x:c r="N42" s="14"/>
+      <x:c r="O42" s="14" t="str">
+        <x:v>Diesel particulate filter</x:v>
+      </x:c>
+      <x:c r="P42" s="14" t="str">
+        <x:v>Permitted / described</x:v>
+      </x:c>
+      <x:c r="Q42" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R42" s="14" t="str">
+        <x:v>OCR pattern extraction</x:v>
+      </x:c>
+      <x:c r="S42" s="14" t="str">
+        <x:v>OCR extracted - review recommended</x:v>
+      </x:c>
+      <x:c r="T42" s="13" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="U42" s="14" t="str">
         <x:v>mittee to CONSTRUCT emission source(s) and/or air pollution control equipment consisting of: Thirty-nine (39) 3,250 kW (4,656 BHP) Diesel-Powered Emergency Generators (Gen1 - Gen39) with 20 Generators equipped with Diesel Particulate Filters (DPFs) ; as descr...</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G2:G39">
+  <x:conditionalFormatting sqref="G2:G42">
     <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Latest operating"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="S2:S39">
+  <x:conditionalFormatting sqref="S2:S42">
     <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="review recommended"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="S2:S39">
+    <x:dataValidation type="list" sqref="S2:S42">
       <x:formula1>"OCR extracted - review recommended,Reviewed,Rejected"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8c9734850444961"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1595208f010f4bb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15714,7 +15900,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd078ca9ff7547ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref781ebee1254388"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16160,7 +16346,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R353365001eba4e39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e4c4d3ba18e4b53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>